<commit_message>
data(figat7th): reconciled pricing + 13-slide test updates
Replaces the FIGat7th scope worksheet with the reconciled pricing pass
and updates golden values + slide-count assertions to match:

  Canopy rental         $22,400        →  $21,197
  Gift Box Trio rental  $4,000-$6,000  →  $3,997-$5,997
  Program ROM rental    $227,150-...   →  $231,527-$239,652
  Program ROM one-time  $280,000-...   →  $299,601-$309,201
  Program ROM service   $117,000-...   →  $107,001-$112,401

Also lifts the four FIGat7th deck-shape assertions from 12 to 13 slides
to reflect the tree_comparison page wired in 4869cd8, and extends the
expected-layout list in test_figat7th_slide_layouts_in_order.

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Projects/Fig at 7th - 2026 - Multi-Rendering Project/03 - Scope & Pricing/FIGat7th DTLA - Scope Worksheet.xlsx
+++ b/Projects/Fig at 7th - 2026 - Multi-Rendering Project/03 - Scope & Pricing/FIGat7th DTLA - Scope Worksheet.xlsx
@@ -655,22 +655,22 @@
       </c>
       <c r="E12" s="6" t="inlineStr"/>
       <c r="F12" s="7" t="n">
-        <v>22400</v>
+        <v>21197</v>
       </c>
       <c r="G12" s="7" t="n">
-        <v>22400</v>
+        <v>21197</v>
       </c>
       <c r="H12" s="7" t="n">
-        <v>19200</v>
+        <v>19197</v>
       </c>
       <c r="I12" s="7" t="n">
-        <v>19200</v>
+        <v>19197</v>
       </c>
       <c r="J12" s="7" t="n">
-        <v>18600</v>
+        <v>17097</v>
       </c>
       <c r="K12" s="7" t="n">
-        <v>18600</v>
+        <v>18597</v>
       </c>
       <c r="L12" s="6" t="inlineStr">
         <is>
@@ -723,22 +723,22 @@
       </c>
       <c r="E14" s="6" t="inlineStr"/>
       <c r="F14" s="7" t="n">
-        <v>150000</v>
+        <v>158623</v>
       </c>
       <c r="G14" s="7" t="n">
-        <v>150000</v>
+        <v>158623</v>
       </c>
       <c r="H14" s="7" t="n">
-        <v>200000</v>
+        <v>222497</v>
       </c>
       <c r="I14" s="7" t="n">
-        <v>200000</v>
+        <v>222497</v>
       </c>
       <c r="J14" s="7" t="n">
-        <v>80000</v>
+        <v>71522</v>
       </c>
       <c r="K14" s="7" t="n">
-        <v>80000</v>
+        <v>71522</v>
       </c>
       <c r="L14" s="6" t="inlineStr">
         <is>
@@ -780,22 +780,22 @@
       </c>
       <c r="E15" s="6" t="inlineStr"/>
       <c r="F15" s="7" t="n">
-        <v>15000</v>
+        <v>14997</v>
       </c>
       <c r="G15" s="7" t="n">
-        <v>15000</v>
+        <v>14997</v>
       </c>
       <c r="H15" s="7" t="n">
-        <v>12000</v>
+        <v>11997</v>
       </c>
       <c r="I15" s="7" t="n">
-        <v>12000</v>
+        <v>11997</v>
       </c>
       <c r="J15" s="7" t="n">
-        <v>5900</v>
+        <v>5897</v>
       </c>
       <c r="K15" s="7" t="n">
-        <v>5900</v>
+        <v>5897</v>
       </c>
       <c r="L15" s="6" t="inlineStr">
         <is>
@@ -848,22 +848,22 @@
         </is>
       </c>
       <c r="F17" s="7" t="n">
-        <v>9500</v>
+        <v>8947</v>
       </c>
       <c r="G17" s="7" t="n">
-        <v>9500</v>
+        <v>9622</v>
       </c>
       <c r="H17" s="7" t="n">
-        <v>9000</v>
+        <v>8997</v>
       </c>
       <c r="I17" s="7" t="n">
-        <v>9000</v>
+        <v>8997</v>
       </c>
       <c r="J17" s="7" t="n">
-        <v>2000</v>
+        <v>2247</v>
       </c>
       <c r="K17" s="7" t="n">
-        <v>2000</v>
+        <v>2247</v>
       </c>
       <c r="L17" s="6" t="inlineStr">
         <is>
@@ -913,22 +913,22 @@
         </is>
       </c>
       <c r="F18" s="7" t="n">
-        <v>9000</v>
+        <v>8997</v>
       </c>
       <c r="G18" s="7" t="n">
-        <v>9000</v>
+        <v>8997</v>
       </c>
       <c r="H18" s="7" t="n">
-        <v>8900</v>
+        <v>8897</v>
       </c>
       <c r="I18" s="7" t="n">
-        <v>8900</v>
+        <v>8897</v>
       </c>
       <c r="J18" s="7" t="n">
-        <v>2000</v>
+        <v>1997</v>
       </c>
       <c r="K18" s="7" t="n">
-        <v>2000</v>
+        <v>1997</v>
       </c>
       <c r="L18" s="6" t="inlineStr">
         <is>
@@ -978,22 +978,22 @@
         </is>
       </c>
       <c r="F19" s="7" t="n">
-        <v>8500</v>
+        <v>7872</v>
       </c>
       <c r="G19" s="7" t="n">
-        <v>8500</v>
+        <v>7872</v>
       </c>
       <c r="H19" s="7" t="n">
-        <v>9500</v>
+        <v>9247</v>
       </c>
       <c r="I19" s="7" t="n">
-        <v>9500</v>
+        <v>9247</v>
       </c>
       <c r="J19" s="7" t="n">
-        <v>2200</v>
+        <v>2197</v>
       </c>
       <c r="K19" s="7" t="n">
-        <v>2200</v>
+        <v>2197</v>
       </c>
       <c r="L19" s="6" t="inlineStr">
         <is>
@@ -1043,22 +1043,22 @@
         </is>
       </c>
       <c r="F20" s="7" t="n">
-        <v>14000</v>
+        <v>13997</v>
       </c>
       <c r="G20" s="7" t="n">
-        <v>14000</v>
+        <v>13997</v>
       </c>
       <c r="H20" s="7" t="n">
-        <v>16500</v>
+        <v>16497</v>
       </c>
       <c r="I20" s="7" t="n">
-        <v>16500</v>
+        <v>16497</v>
       </c>
       <c r="J20" s="7" t="n">
-        <v>2900</v>
+        <v>2897</v>
       </c>
       <c r="K20" s="7" t="n">
-        <v>2900</v>
+        <v>2897</v>
       </c>
       <c r="L20" s="6" t="inlineStr">
         <is>
@@ -1111,22 +1111,22 @@
       </c>
       <c r="E22" s="6" t="inlineStr"/>
       <c r="F22" s="7" t="n">
-        <v>9500</v>
+        <v>7997</v>
       </c>
       <c r="G22" s="7" t="n">
-        <v>9500</v>
+        <v>7997</v>
       </c>
       <c r="H22" s="7" t="n">
-        <v>12000</v>
+        <v>10247</v>
       </c>
       <c r="I22" s="7" t="n">
-        <v>12000</v>
+        <v>10247</v>
       </c>
       <c r="J22" s="7" t="n">
-        <v>2500</v>
+        <v>2497</v>
       </c>
       <c r="K22" s="7" t="n">
-        <v>2500</v>
+        <v>2497</v>
       </c>
       <c r="L22" s="6" t="inlineStr">
         <is>
@@ -1168,22 +1168,22 @@
       </c>
       <c r="E23" s="6" t="inlineStr"/>
       <c r="F23" s="7" t="n">
-        <v>10250</v>
+        <v>9347</v>
       </c>
       <c r="G23" s="7" t="n">
-        <v>10250</v>
+        <v>9347</v>
       </c>
       <c r="H23" s="7" t="n">
-        <v>12500</v>
+        <v>11372</v>
       </c>
       <c r="I23" s="7" t="n">
-        <v>12500</v>
+        <v>11372</v>
       </c>
       <c r="J23" s="7" t="n">
-        <v>2500</v>
+        <v>2497</v>
       </c>
       <c r="K23" s="7" t="n">
-        <v>2500</v>
+        <v>2497</v>
       </c>
       <c r="L23" s="6" t="inlineStr">
         <is>
@@ -1225,22 +1225,22 @@
       </c>
       <c r="E24" s="6" t="inlineStr"/>
       <c r="F24" s="7" t="n">
-        <v>7500</v>
+        <v>7497</v>
       </c>
       <c r="G24" s="7" t="n">
-        <v>7500</v>
+        <v>7497</v>
       </c>
       <c r="H24" s="7" t="n">
-        <v>9400</v>
+        <v>9397</v>
       </c>
       <c r="I24" s="7" t="n">
-        <v>9400</v>
+        <v>9397</v>
       </c>
       <c r="J24" s="7" t="n">
-        <v>1500</v>
+        <v>1497</v>
       </c>
       <c r="K24" s="7" t="n">
-        <v>1500</v>
+        <v>1497</v>
       </c>
       <c r="L24" s="6" t="inlineStr">
         <is>
@@ -1282,22 +1282,22 @@
       </c>
       <c r="E25" s="6" t="inlineStr"/>
       <c r="F25" s="7" t="n">
-        <v>4000</v>
+        <v>3997</v>
       </c>
       <c r="G25" s="7" t="n">
-        <v>6000</v>
+        <v>5997</v>
       </c>
       <c r="H25" s="7" t="n">
-        <v>6000</v>
+        <v>5997</v>
       </c>
       <c r="I25" s="7" t="n">
-        <v>8000</v>
+        <v>7997</v>
       </c>
       <c r="J25" s="7" t="n">
-        <v>4000</v>
+        <v>3997</v>
       </c>
       <c r="K25" s="7" t="n">
-        <v>7000</v>
+        <v>6997</v>
       </c>
       <c r="L25" s="6" t="inlineStr">
         <is>

</xml_diff>